<commit_message>
data driven testing by excel file
</commit_message>
<xml_diff>
--- a/src/test/java/CompeteHealth/TestData/Logindata.xlsx
+++ b/src/test/java/CompeteHealth/TestData/Logindata.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="6" lowestEdited="4" rupBuild="14420"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="124226"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="15885" windowHeight="3465"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="15885" windowHeight="3720"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="6">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10" uniqueCount="7">
   <si>
     <t>user</t>
   </si>
@@ -33,13 +33,16 @@
   </si>
   <si>
     <t>demo@yopmail.com</t>
+  </si>
+  <si>
+    <t>triumpco5@yopmail.com</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -54,6 +57,12 @@
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color rgb="FF212529"/>
+      <name val="Segoe UI"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="2">
@@ -77,7 +86,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
@@ -85,6 +94,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -390,7 +400,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:B4"/>
+  <dimension ref="A1:B5"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="28.7109375" style="1" customWidth="1"/>
@@ -406,7 +416,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:2" s="1" customFormat="1" ht="45" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:2" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
         <v>2</v>
       </c>
@@ -427,6 +437,14 @@
         <v>5</v>
       </c>
       <c r="B4" s="2" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" ht="17.25" x14ac:dyDescent="0.3">
+      <c r="A5" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="B5" s="2" t="s">
         <v>3</v>
       </c>
     </row>
@@ -438,7 +456,9 @@
     <hyperlink ref="B3" r:id="rId4"/>
     <hyperlink ref="A4" r:id="rId5"/>
     <hyperlink ref="B4" r:id="rId6"/>
+    <hyperlink ref="B5" r:id="rId7"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId8"/>
 </worksheet>
 </file>
</xml_diff>